<commit_message>
Lançar o programa de metas de setembro e manter o PEDRO em R$ 1.621
Nova aba METAS SET.26 em cada loja, a partir da planilha
Metas_Equipe_Set2026_v2.xlsx: meta individual, faixa, dias trabalhados,
meta ajustada e o prêmio de cada uma das 4 metas (volume, produtos
foco, pré-vencidos e perfumaria 130% da loja), com as regras próprias
dos farmacêuticos e o acordo à parte de DEAN e AGNOR na Meta 1.

No holerite, as linhas de prêmio passam a ser uma por meta e puxam o
valor da aba METAS. Os prêmios aparecem quando as vendas de setembro
forem lançadas.

PEDRO segue com R$ 1.621,00 no pagamento de 05/10; os R$ 4.000,00
começam na competência de outubro. Remove o __pycache__ do controle de
versão.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RESUMO_3_LOJAS_SETEMBRO_2026_pgto_05-10-2026.xlsx
+++ b/relatorios/contabilidade/RESUMO_3_LOJAS_SETEMBRO_2026_pgto_05-10-2026.xlsx
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W44"/>
+  <dimension ref="A1:W45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>4000</v>
+        <v>1621</v>
       </c>
       <c r="C21" s="7" t="n">
         <v>0</v>
@@ -1904,7 +1904,7 @@
       <c r="V21" s="10" t="n"/>
       <c r="W21" s="11" t="inlineStr">
         <is>
-          <t>Registrado na matriz. Salário corrigido para R$ 4.000,00. Não recebe comissão. O holerite de agosto dele não veio da Betel — pedir junto.</t>
+          <t>Registrado na matriz. Nesta folha segue com R$ 1.621,00; o salário de R$ 4.000,00 começa na competência de outubro (pagamento 05/11). Não recebe comissão. O holerite de agosto dele não veio da Betel — pedir junto.</t>
         </is>
       </c>
     </row>
@@ -2602,77 +2602,85 @@
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>• Prêmios (cota geral e pré-vencidos), vales adiantados, convênio e faltas — por enquanto só o adiantamento do GENECIR está lançado.</t>
+          <t>• Prêmios do programa de metas de setembro (Metas 1 a 4): as metas de cada um já estão na aba METAS SET.26 de cada loja; os prêmios saem sozinhos quando a venda realizada, o pré-vencido vendido, a Meta 2 e a perfumaria da loja forem lançados.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="19" t="inlineStr">
         <is>
-          <t>• Ponto de setembro: horas extras e quem mais trabalhou nos feriados de 07/09 e 08/09.</t>
+          <t>• Vales adiantados, convênio e faltas — por enquanto só o adiantamento do GENECIR está lançado.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="19" t="inlineStr">
         <is>
-          <t>• INSS e IRRF são calculados pela Betel.</t>
+          <t>• Ponto de setembro: horas extras e quem mais trabalhou nos feriados de 07/09 e 08/09.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="19" t="inlineStr">
         <is>
+          <t>• INSS e IRRF são calculados pela Betel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
           <t>• Diárias dos folguistas SERGIO e ANA CELIA (contas a pagar, fora do holerite).</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="19" t="inlineStr"/>
-    </row>
     <row r="40">
-      <c r="A40" s="18" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>CRITÉRIOS DE SETEMBRO:</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="19" t="inlineStr">
-        <is>
-          <t>• DSR: 4 domingos + feriados de 07/09 (Independência) e 08/09 (municipal) = 6 ÷ 24 dias úteis = fator 0,25.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="19" t="inlineStr">
         <is>
-          <t>• Feriado trabalhado sem folga = 1 salário-dia a mais (R$ 54,03 no salário de R$ 1.621,00).</t>
+          <t>• DSR: 4 domingos + feriados de 07/09 (Independência) e 08/09 (municipal) = 6 ÷ 24 dias úteis = fator 0,25.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="19" t="inlineStr">
         <is>
-          <t>• TRANCOSO paga o dobro da comissão apurada; incentivos simples.</t>
+          <t>• Feriado trabalhado sem folga = 1 salário-dia a mais (R$ 54,03 no salário de R$ 1.621,00).</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="19" t="inlineStr">
         <is>
+          <t>• TRANCOSO paga o dobro da comissão apurada; incentivos simples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
           <t>• Férias pagas à parte em setembro: RENALDO (Centro) e VALDICK (Trancoso), de 01 a 30/09 — lançar o valor do recibo na coluna FÉRIAS PAGAS À PARTE.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:W29"/>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="A36:W36"/>
     <mergeCell ref="A44:W44"/>
     <mergeCell ref="A1:W1"/>
     <mergeCell ref="A37:W37"/>
     <mergeCell ref="A40:W40"/>
+    <mergeCell ref="A45:W45"/>
     <mergeCell ref="A34:W34"/>
     <mergeCell ref="A35:W35"/>
     <mergeCell ref="A38:W38"/>

</xml_diff>